<commit_message>
Fix theoretical close mode and update Excel
</commit_message>
<xml_diff>
--- a/MinusLock_Self_Compressing_Recovery_Calculator/MinusLock_Self_Compressing_Recovery_Calculator.xlsx
+++ b/MinusLock_Self_Compressing_Recovery_Calculator/MinusLock_Self_Compressing_Recovery_Calculator.xlsx
@@ -421,11 +421,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP44"/>
+  <dimension ref="A1:AQ45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ПАРАМЕТРЫ</t>
         </is>
@@ -516,11 +516,13 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>UseProfitReserveClose</t>
-        </is>
-      </c>
-      <c r="B10" t="b">
-        <v>1</v>
+          <t>CloseMode</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>THEORETICAL</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -640,257 +642,218 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="n"/>
-      <c r="B25" s="1" t="n"/>
-      <c r="C25" s="1" t="n"/>
-      <c r="D25" s="1" t="n"/>
-      <c r="E25" s="1" t="n"/>
-      <c r="F25" s="1" t="n"/>
-      <c r="G25" s="1" t="n"/>
-      <c r="H25" s="1" t="n"/>
-      <c r="I25" s="1" t="n"/>
-      <c r="J25" s="1" t="n"/>
-      <c r="K25" s="1" t="n"/>
-      <c r="L25" s="1" t="n"/>
-      <c r="M25" s="1" t="n"/>
-      <c r="N25" s="1" t="n"/>
-      <c r="O25" s="1" t="n"/>
-      <c r="P25" s="1" t="n"/>
-      <c r="Q25" s="1" t="n"/>
-      <c r="R25" s="1" t="n"/>
-      <c r="S25" s="1" t="n"/>
-      <c r="T25" s="1" t="n"/>
-      <c r="U25" s="1" t="n"/>
-      <c r="V25" s="1" t="n"/>
-      <c r="W25" s="1" t="n"/>
-      <c r="X25" s="1" t="n"/>
-      <c r="Y25" s="1" t="n"/>
-      <c r="Z25" s="1" t="n"/>
-      <c r="AA25" s="1" t="n"/>
-      <c r="AB25" s="1" t="n"/>
-      <c r="AC25" s="1" t="n"/>
-      <c r="AD25" s="1" t="n"/>
-      <c r="AE25" s="1" t="n"/>
-      <c r="AF25" s="1" t="n"/>
-      <c r="AG25" s="1" t="n"/>
-      <c r="AH25" s="1" t="n"/>
-      <c r="AI25" s="1" t="n"/>
-      <c r="AJ25" s="1" t="n"/>
-      <c r="AK25" s="1" t="n"/>
-      <c r="AL25" s="1" t="n"/>
-      <c r="AM25" s="1" t="n"/>
-      <c r="AN25" s="1" t="n"/>
-      <c r="AO25" s="1" t="n"/>
-      <c r="AP25" s="1" t="n"/>
-    </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>Уровень</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>Направление</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>Ближний старт</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="1" t="inlineStr">
         <is>
           <t>Дальний старт остаток</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="1" t="inlineStr">
         <is>
           <t>Старт поз. самая дальняя</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="1" t="inlineStr">
         <is>
           <t>Big %</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="1" t="inlineStr">
         <is>
           <t>Big Lot Raw</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H26" s="1" t="inlineStr">
         <is>
           <t>Big Lot Rounded</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I26" s="1" t="inlineStr">
         <is>
           <t>Small %</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J26" s="1" t="inlineStr">
         <is>
           <t>Small Lot Raw</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K26" s="1" t="inlineStr">
         <is>
           <t>Small Lot Rounded</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="L26" s="1" t="inlineStr">
         <is>
           <t>Close Far %</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="M26" s="1" t="inlineStr">
         <is>
           <t>Max Close Far Lot</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="N26" s="1" t="inlineStr">
+        <is>
+          <t>Close By Profit Budget</t>
+        </is>
+      </c>
+      <c r="O26" s="1" t="inlineStr">
         <is>
           <t>Actual Close Far Lot</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
+      <c r="P26" s="1" t="inlineStr">
+        <is>
+          <t>Close Mode</t>
+        </is>
+      </c>
+      <c r="Q26" s="1" t="inlineStr">
         <is>
           <t>Новый ближний старт</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
+      <c r="R26" s="1" t="inlineStr">
         <is>
           <t>Новый дальний остаток</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr">
+      <c r="S26" s="1" t="inlineStr">
         <is>
           <t>Next Base Lot</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
+      <c r="T26" s="1" t="inlineStr">
         <is>
           <t>Сумма Big</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr">
+      <c r="U26" s="1" t="inlineStr">
         <is>
           <t>Сумма Small</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr">
+      <c r="V26" s="1" t="inlineStr">
         <is>
           <t>Сумма Close</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="W26" s="1" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="V26" t="inlineStr">
+      <c r="X26" s="1" t="inlineStr">
         <is>
           <t>Комментарий</t>
         </is>
       </c>
-      <c r="W26" t="inlineStr">
+      <c r="Y26" s="1" t="inlineStr">
         <is>
           <t>Прибыль пакета до Close</t>
         </is>
       </c>
-      <c r="X26" t="inlineStr">
+      <c r="Z26" s="1" t="inlineStr">
         <is>
           <t>Резерв %</t>
         </is>
       </c>
-      <c r="Y26" t="inlineStr">
+      <c r="AA26" s="1" t="inlineStr">
         <is>
           <t>Резерв деньги</t>
         </is>
       </c>
-      <c r="Z26" t="inlineStr">
+      <c r="AB26" s="1" t="inlineStr">
         <is>
           <t>Бюджет на Close</t>
         </is>
       </c>
-      <c r="AA26" t="inlineStr">
+      <c r="AC26" s="1" t="inlineStr">
         <is>
           <t>Убыток Far Start на 1 лот</t>
         </is>
       </c>
-      <c r="AB26" t="inlineStr">
-        <is>
-          <t>Close по бюджету</t>
-        </is>
-      </c>
-      <c r="AC26" t="inlineStr">
+      <c r="AD26" s="1" t="inlineStr">
         <is>
           <t>Остаток резерва после Close</t>
         </is>
       </c>
-      <c r="AD26" t="inlineStr">
+      <c r="AE26" s="1" t="inlineStr">
         <is>
           <t>Close Status</t>
         </is>
       </c>
-      <c r="AE26" t="inlineStr">
+      <c r="AF26" s="1" t="inlineStr">
         <is>
           <t>Total Big Lots</t>
         </is>
       </c>
-      <c r="AF26" t="inlineStr">
+      <c r="AG26" s="1" t="inlineStr">
         <is>
           <t>Total Small Lots</t>
         </is>
       </c>
-      <c r="AG26" t="inlineStr">
+      <c r="AH26" s="1" t="inlineStr">
         <is>
           <t>Total Open Lots</t>
         </is>
       </c>
-      <c r="AH26" t="inlineStr">
+      <c r="AI26" s="1" t="inlineStr">
         <is>
           <t>Net Lot</t>
         </is>
       </c>
-      <c r="AI26" t="inlineStr">
+      <c r="AJ26" s="1" t="inlineStr">
         <is>
           <t>Margin Per Lot</t>
         </is>
       </c>
-      <c r="AJ26" t="inlineStr">
+      <c r="AK26" s="1" t="inlineStr">
         <is>
           <t>Required Margin</t>
         </is>
       </c>
-      <c r="AK26" t="inlineStr">
+      <c r="AL26" s="1" t="inlineStr">
         <is>
           <t>Margin Load %</t>
         </is>
       </c>
-      <c r="AL26" t="inlineStr">
+      <c r="AM26" s="1" t="inlineStr">
         <is>
           <t>Floating DD</t>
         </is>
       </c>
-      <c r="AM26" t="inlineStr">
+      <c r="AN26" s="1" t="inlineStr">
         <is>
           <t>Equity After DD</t>
         </is>
       </c>
-      <c r="AN26" t="inlineStr">
+      <c r="AO26" s="1" t="inlineStr">
         <is>
           <t>Free Margin</t>
         </is>
       </c>
-      <c r="AO26" t="inlineStr">
+      <c r="AP26" s="1" t="inlineStr">
         <is>
           <t>Margin Level %</t>
         </is>
       </c>
-      <c r="AP26" t="inlineStr">
+      <c r="AQ26" s="1" t="inlineStr">
         <is>
           <t>Risk Status</t>
         </is>
@@ -944,93 +907,98 @@
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P27" t="n">
-        <v>1</v>
+        <v>0.3</v>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>THEORETICAL</t>
+        </is>
       </c>
       <c r="Q27" t="n">
         <v>0.5</v>
       </c>
       <c r="R27" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="S27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T27" t="n">
         <v>0.9</v>
       </c>
-      <c r="S27" t="n">
+      <c r="U27" t="n">
         <v>0.4</v>
       </c>
-      <c r="T27" t="n">
+      <c r="V27" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>Уровень 1. Цена идёт вниз. Ближний старт=1.00000. Открыть Big BUY 0.90000. Открыть Small SELL 0.40000. Частично закрыть дальний Start BUY 0.30000. Новый ближний старт=0.50000. Остаток дальнего Start BUY=0.70000. Статус=OK.</t>
+        </is>
+      </c>
+      <c r="Y27" t="n">
+        <v>13</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>30</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB27" t="n">
+        <v>8</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AD27" t="n">
         <v>0</v>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="AE27" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>Уровень 1. Цена идёт вниз. Ближний старт=1.00000. Открыть Big BUY 0.90000. Открыть Small SELL 0.40000. Частично закрыть дальний Start BUY 0.00000. Новый ближний старт=0.50000. Остаток дальнего Start BUY=1.00000. Статус=OK.</t>
-        </is>
-      </c>
-      <c r="W27" t="n">
-        <v>13</v>
-      </c>
-      <c r="X27" t="n">
-        <v>30</v>
-      </c>
-      <c r="Y27" t="n">
-        <v>5</v>
-      </c>
-      <c r="Z27" t="n">
-        <v>8</v>
-      </c>
-      <c r="AA27" t="n">
-        <v>5000</v>
-      </c>
-      <c r="AB27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC27" t="n">
-        <v>13</v>
-      </c>
-      <c r="AD27" t="inlineStr">
-        <is>
-          <t>NO CLOSE</t>
-        </is>
-      </c>
-      <c r="AE27" t="n">
+      <c r="AF27" t="n">
         <v>0.9</v>
       </c>
-      <c r="AF27" t="n">
+      <c r="AG27" t="n">
         <v>0.4</v>
       </c>
-      <c r="AG27" t="n">
+      <c r="AH27" t="n">
         <v>1.3</v>
       </c>
-      <c r="AH27" t="n">
+      <c r="AI27" t="n">
         <v>0.5</v>
       </c>
-      <c r="AI27" t="n">
+      <c r="AJ27" t="n">
         <v>1100</v>
       </c>
-      <c r="AJ27" t="n">
+      <c r="AK27" t="n">
         <v>1430</v>
       </c>
-      <c r="AK27" t="n">
+      <c r="AL27" t="n">
         <v>14.3</v>
       </c>
-      <c r="AL27" t="n">
+      <c r="AM27" t="n">
         <v>2500</v>
       </c>
-      <c r="AM27" t="n">
+      <c r="AN27" t="n">
         <v>7500</v>
       </c>
-      <c r="AN27" t="n">
+      <c r="AO27" t="n">
         <v>6070</v>
       </c>
-      <c r="AO27" t="n">
+      <c r="AP27" t="n">
         <v>524.4755244755244</v>
       </c>
-      <c r="AP27" t="inlineStr">
+      <c r="AQ27" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1049,7 +1017,7 @@
         <v>0.5</v>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1084,93 +1052,98 @@
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="P28" t="n">
-        <v>1</v>
+        <v>0.15</v>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>THEORETICAL</t>
+        </is>
       </c>
       <c r="Q28" t="n">
         <v>0.25</v>
       </c>
       <c r="R28" t="n">
+        <v>0.5499999999999999</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="T28" t="n">
         <v>1.35</v>
       </c>
-      <c r="S28" t="n">
+      <c r="U28" t="n">
         <v>0.6000000000000001</v>
       </c>
-      <c r="T28" t="n">
+      <c r="V28" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>Уровень 2. Цена идёт вниз. Ближний старт=0.50000. Открыть Big BUY 0.45000. Открыть Small SELL 0.20000. Частично закрыть дальний Start BUY 0.15000. Новый ближний старт=0.25000. Остаток дальнего Start BUY=0.55000. Статус=OK.</t>
+        </is>
+      </c>
+      <c r="Y28" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>30</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB28" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AD28" t="n">
         <v>0</v>
       </c>
-      <c r="U28" t="inlineStr">
+      <c r="AE28" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>Уровень 2. Цена идёт вниз. Ближний старт=0.50000. Открыть Big BUY 0.45000. Открыть Small SELL 0.20000. Частично закрыть дальний Start BUY 0.00000. Новый ближний старт=0.25000. Остаток дальнего Start BUY=1.00000. Статус=OK.</t>
-        </is>
-      </c>
-      <c r="W28" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="X28" t="n">
-        <v>30</v>
-      </c>
-      <c r="Y28" t="n">
-        <v>5</v>
-      </c>
-      <c r="Z28" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="AA28" t="n">
-        <v>5000</v>
-      </c>
-      <c r="AB28" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC28" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="AD28" t="inlineStr">
-        <is>
-          <t>NO CLOSE</t>
-        </is>
-      </c>
-      <c r="AE28" t="n">
+      <c r="AF28" t="n">
         <v>1.35</v>
       </c>
-      <c r="AF28" t="n">
+      <c r="AG28" t="n">
         <v>0.6000000000000001</v>
       </c>
-      <c r="AG28" t="n">
+      <c r="AH28" t="n">
         <v>1.95</v>
       </c>
-      <c r="AH28" t="n">
+      <c r="AI28" t="n">
         <v>0.75</v>
       </c>
-      <c r="AI28" t="n">
+      <c r="AJ28" t="n">
         <v>1100</v>
       </c>
-      <c r="AJ28" t="n">
+      <c r="AK28" t="n">
         <v>2145</v>
       </c>
-      <c r="AK28" t="n">
+      <c r="AL28" t="n">
         <v>21.45000000000001</v>
       </c>
-      <c r="AL28" t="n">
+      <c r="AM28" t="n">
         <v>3750</v>
       </c>
-      <c r="AM28" t="n">
+      <c r="AN28" t="n">
         <v>6250</v>
       </c>
-      <c r="AN28" t="n">
+      <c r="AO28" t="n">
         <v>4105</v>
       </c>
-      <c r="AO28" t="n">
+      <c r="AP28" t="n">
         <v>291.3752913752913</v>
       </c>
-      <c r="AP28" t="inlineStr">
+      <c r="AQ28" t="inlineStr">
         <is>
           <t>WARNING</t>
         </is>
@@ -1189,7 +1162,7 @@
         <v>0.25</v>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>0.5499999999999999</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1224,93 +1197,98 @@
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="P29" t="n">
-        <v>1</v>
+        <v>0.075</v>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>THEORETICAL</t>
+        </is>
       </c>
       <c r="Q29" t="n">
-        <v>0.13</v>
+        <v>0.125</v>
       </c>
       <c r="R29" t="n">
+        <v>0.4749999999999999</v>
+      </c>
+      <c r="S29" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="T29" t="n">
         <v>1.57</v>
       </c>
-      <c r="S29" t="n">
+      <c r="U29" t="n">
         <v>0.7000000000000001</v>
       </c>
-      <c r="T29" t="n">
+      <c r="V29" t="n">
+        <v>0.5249999999999999</v>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>Уровень 3. Цена идёт вниз. Ближний старт=0.25000. Открыть Big BUY 0.22000. Открыть Small SELL 0.10000. Частично закрыть дальний Start BUY 0.07500. Новый ближний старт=0.12500. Остаток дальнего Start BUY=0.47500. Статус=OK.</t>
+        </is>
+      </c>
+      <c r="Y29" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>30</v>
+      </c>
+      <c r="AA29" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB29" t="n">
+        <v>-1.8</v>
+      </c>
+      <c r="AC29" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AD29" t="n">
         <v>0</v>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="AE29" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>Уровень 3. Цена идёт вниз. Ближний старт=0.25000. Открыть Big BUY 0.22000. Открыть Small SELL 0.10000. Частично закрыть дальний Start BUY 0.00000. Новый ближний старт=0.13000. Остаток дальнего Start BUY=1.00000. Статус=OK.</t>
-        </is>
-      </c>
-      <c r="W29" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="X29" t="n">
-        <v>30</v>
-      </c>
-      <c r="Y29" t="n">
-        <v>5</v>
-      </c>
-      <c r="Z29" t="n">
-        <v>-1.8</v>
-      </c>
-      <c r="AA29" t="n">
-        <v>5000</v>
-      </c>
-      <c r="AB29" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC29" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="AD29" t="inlineStr">
-        <is>
-          <t>NO CLOSE</t>
-        </is>
-      </c>
-      <c r="AE29" t="n">
+      <c r="AF29" t="n">
         <v>1.57</v>
       </c>
-      <c r="AF29" t="n">
+      <c r="AG29" t="n">
         <v>0.7000000000000001</v>
       </c>
-      <c r="AG29" t="n">
+      <c r="AH29" t="n">
         <v>2.27</v>
       </c>
-      <c r="AH29" t="n">
+      <c r="AI29" t="n">
         <v>0.87</v>
       </c>
-      <c r="AI29" t="n">
+      <c r="AJ29" t="n">
         <v>1100</v>
       </c>
-      <c r="AJ29" t="n">
+      <c r="AK29" t="n">
         <v>2497</v>
       </c>
-      <c r="AK29" t="n">
+      <c r="AL29" t="n">
         <v>24.97</v>
       </c>
-      <c r="AL29" t="n">
+      <c r="AM29" t="n">
         <v>4350</v>
       </c>
-      <c r="AM29" t="n">
+      <c r="AN29" t="n">
         <v>5650</v>
       </c>
-      <c r="AN29" t="n">
+      <c r="AO29" t="n">
         <v>3153</v>
       </c>
-      <c r="AO29" t="n">
+      <c r="AP29" t="n">
         <v>226.2715258309972</v>
       </c>
-      <c r="AP29" t="inlineStr">
+      <c r="AQ29" t="inlineStr">
         <is>
           <t>WARNING</t>
         </is>
@@ -1326,10 +1304,10 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.13</v>
+        <v>0.125</v>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>0.4749999999999999</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1340,7 +1318,7 @@
         <v>90</v>
       </c>
       <c r="G30" t="n">
-        <v>0.117</v>
+        <v>0.1125</v>
       </c>
       <c r="H30" t="n">
         <v>0.11</v>
@@ -1349,108 +1327,113 @@
         <v>40</v>
       </c>
       <c r="J30" t="n">
-        <v>0.052</v>
+        <v>0.05</v>
       </c>
       <c r="K30" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="L30" t="n">
         <v>30</v>
       </c>
       <c r="M30" t="n">
-        <v>0.03900000000000001</v>
+        <v>0.0375</v>
       </c>
       <c r="N30" t="n">
         <v>0</v>
       </c>
       <c r="O30" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="P30" t="n">
-        <v>1</v>
+        <v>0.0375</v>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>THEORETICAL</t>
+        </is>
       </c>
       <c r="Q30" t="n">
-        <v>0.08</v>
+        <v>0.0625</v>
       </c>
       <c r="R30" t="n">
+        <v>0.4374999999999999</v>
+      </c>
+      <c r="S30" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="T30" t="n">
         <v>1.68</v>
       </c>
-      <c r="S30" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="T30" t="n">
+      <c r="U30" t="n">
+        <v>0.7500000000000001</v>
+      </c>
+      <c r="V30" t="n">
+        <v>0.5624999999999999</v>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>Уровень 4. Цена идёт вниз. Ближний старт=0.12500. Открыть Big BUY 0.11000. Открыть Small SELL 0.05000. Частично закрыть дальний Start BUY 0.03750. Новый ближний старт=0.06250. Остаток дальнего Start BUY=0.43750. Статус=OK.</t>
+        </is>
+      </c>
+      <c r="Y30" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>30</v>
+      </c>
+      <c r="AA30" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB30" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AD30" t="n">
         <v>0</v>
       </c>
-      <c r="U30" t="inlineStr">
+      <c r="AE30" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>Уровень 4. Цена идёт вниз. Ближний старт=0.13000. Открыть Big BUY 0.11000. Открыть Small SELL 0.06000. Частично закрыть дальний Start BUY 0.00000. Новый ближний старт=0.08000. Остаток дальнего Start BUY=1.00000. Статус=OK.</t>
-        </is>
-      </c>
-      <c r="W30" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="X30" t="n">
-        <v>30</v>
-      </c>
-      <c r="Y30" t="n">
-        <v>5</v>
-      </c>
-      <c r="Z30" t="n">
-        <v>-3.3</v>
-      </c>
-      <c r="AA30" t="n">
-        <v>5000</v>
-      </c>
-      <c r="AB30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC30" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="AD30" t="inlineStr">
-        <is>
-          <t>NO CLOSE</t>
-        </is>
-      </c>
-      <c r="AE30" t="n">
+      <c r="AF30" t="n">
         <v>1.68</v>
       </c>
-      <c r="AF30" t="n">
-        <v>0.76</v>
-      </c>
       <c r="AG30" t="n">
-        <v>2.44</v>
+        <v>0.7500000000000001</v>
       </c>
       <c r="AH30" t="n">
-        <v>0.9200000000000002</v>
+        <v>2.43</v>
       </c>
       <c r="AI30" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="AJ30" t="n">
         <v>1100</v>
       </c>
-      <c r="AJ30" t="n">
-        <v>2684.000000000001</v>
-      </c>
       <c r="AK30" t="n">
-        <v>26.84000000000001</v>
+        <v>2673.000000000001</v>
       </c>
       <c r="AL30" t="n">
-        <v>4600.000000000001</v>
+        <v>26.73000000000001</v>
       </c>
       <c r="AM30" t="n">
-        <v>5399.999999999999</v>
+        <v>4650</v>
       </c>
       <c r="AN30" t="n">
-        <v>2715.999999999998</v>
+        <v>5350</v>
       </c>
       <c r="AO30" t="n">
-        <v>201.1922503725781</v>
-      </c>
-      <c r="AP30" t="inlineStr">
+        <v>2676.999999999999</v>
+      </c>
+      <c r="AP30" t="n">
+        <v>200.149644594089</v>
+      </c>
+      <c r="AQ30" t="inlineStr">
         <is>
           <t>WARNING</t>
         </is>
@@ -1466,10 +1449,10 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.08</v>
+        <v>0.0625</v>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>0.4374999999999999</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1480,242 +1463,246 @@
         <v>90</v>
       </c>
       <c r="G31" t="n">
-        <v>0.07200000000000001</v>
+        <v>0.05625</v>
       </c>
       <c r="H31" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.05</v>
       </c>
       <c r="I31" t="n">
         <v>40</v>
       </c>
       <c r="J31" t="n">
-        <v>0.032</v>
+        <v>0.025</v>
       </c>
       <c r="K31" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="L31" t="n">
         <v>30</v>
       </c>
       <c r="M31" t="n">
-        <v>0.024</v>
+        <v>0.01875</v>
       </c>
       <c r="N31" t="n">
         <v>0</v>
       </c>
       <c r="O31" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="P31" t="n">
-        <v>1</v>
+        <v>0.01875</v>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>THEORETICAL</t>
+        </is>
       </c>
       <c r="Q31" t="n">
-        <v>0.05</v>
+        <v>0.03125</v>
       </c>
       <c r="R31" t="n">
-        <v>1.75</v>
+        <v>0.41875</v>
       </c>
       <c r="S31" t="n">
+        <v>0.03125</v>
+      </c>
+      <c r="T31" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="U31" t="n">
+        <v>0.7800000000000001</v>
+      </c>
+      <c r="V31" t="n">
+        <v>0.5812499999999999</v>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>Уровень 5. Цена идёт вниз. Ближний старт=0.06250. Открыть Big BUY 0.05000. Открыть Small SELL 0.03000. Частично закрыть дальний Start BUY 0.01875. Новый ближний старт=0.03125. Остаток дальнего Start BUY=0.41875. Статус=OK.</t>
+        </is>
+      </c>
+      <c r="Y31" t="n">
         <v>0.8</v>
       </c>
-      <c r="T31" t="n">
+      <c r="Z31" t="n">
+        <v>30</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB31" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AD31" t="n">
         <v>0</v>
       </c>
-      <c r="U31" t="inlineStr">
+      <c r="AE31" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>Уровень 5. Цена идёт вниз. Ближний старт=0.08000. Открыть Big BUY 0.07000. Открыть Small SELL 0.04000. Частично закрыть дальний Start BUY 0.00000. Новый ближний старт=0.05000. Остаток дальнего Start BUY=1.00000. Статус=OK.</t>
-        </is>
-      </c>
-      <c r="W31" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="X31" t="n">
-        <v>30</v>
-      </c>
-      <c r="Y31" t="n">
-        <v>5</v>
-      </c>
-      <c r="Z31" t="n">
-        <v>-3.9</v>
-      </c>
-      <c r="AA31" t="n">
-        <v>5000</v>
-      </c>
-      <c r="AB31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC31" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="AD31" t="inlineStr">
-        <is>
-          <t>NO CLOSE</t>
-        </is>
-      </c>
-      <c r="AE31" t="n">
-        <v>1.75</v>
-      </c>
       <c r="AF31" t="n">
-        <v>0.8</v>
+        <v>1.73</v>
       </c>
       <c r="AG31" t="n">
-        <v>2.55</v>
+        <v>0.7800000000000001</v>
       </c>
       <c r="AH31" t="n">
-        <v>0.9500000000000002</v>
+        <v>2.51</v>
       </c>
       <c r="AI31" t="n">
+        <v>0.9500000000000001</v>
+      </c>
+      <c r="AJ31" t="n">
         <v>1100</v>
       </c>
-      <c r="AJ31" t="n">
-        <v>2805.000000000001</v>
-      </c>
       <c r="AK31" t="n">
-        <v>28.05000000000001</v>
+        <v>2761.000000000001</v>
       </c>
       <c r="AL31" t="n">
+        <v>27.61000000000001</v>
+      </c>
+      <c r="AM31" t="n">
         <v>4750.000000000001</v>
       </c>
-      <c r="AM31" t="n">
+      <c r="AN31" t="n">
         <v>5249.999999999999</v>
       </c>
-      <c r="AN31" t="n">
-        <v>2444.999999999998</v>
-      </c>
       <c r="AO31" t="n">
-        <v>187.1657754010694</v>
-      </c>
-      <c r="AP31" t="inlineStr">
+        <v>2488.999999999998</v>
+      </c>
+      <c r="AP31" t="n">
+        <v>190.1484969214052</v>
+      </c>
+      <c r="AQ31" t="inlineStr">
         <is>
           <t>WARNING</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
         <is>
           <t>ИТОГИ САМОСЖИМАЮЩЕЙСЯ МОДЕЛИ</t>
         </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>StartLot</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
+          <t>StartLot</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Финальная сумма Big</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>1.75</v>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Финальная сумма Small</t>
+          <t>Финальная сумма Big</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.8</v>
+        <v>1.73</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Финальная сумма Close Far</t>
+          <t>Финальная сумма Small</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0</v>
+        <v>0.7800000000000001</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Финальный ближний старт</t>
+          <t>Финальная сумма Close Far</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.05</v>
+        <v>0.5812499999999999</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Финальный дальний остаток</t>
+          <t>Финальный ближний старт</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>0.03125</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Финальный NextBaseLot</t>
+          <t>Финальный дальний остаток</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.05</v>
+        <v>0.41875</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Количество уровней OK</t>
-        </is>
-      </c>
-      <c r="B42">
-        <f>COUNTIF(A26:A31,"&gt;0")-COUNTIF(U26:U31,"STOP")</f>
-        <v/>
+          <t>Финальный NextBaseLot</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0.03125</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Количество STOP</t>
-        </is>
-      </c>
-      <c r="B43">
-        <f>COUNTIF(U26:U31,"STOP")</f>
-        <v/>
+          <t>Количество уровней OK</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>Количество STOP</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>Финальный статус системы</t>
         </is>
       </c>
-      <c r="B44">
-        <f>IF(COUNTIF(U26:U31,"STOP")&gt;0,"STOP","OK")</f>
-        <v/>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1729,9 +1716,292 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Уровень</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Total Big Lots</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Total Small Lots</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Total Open Lots</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Net Lot</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Margin Per Lot</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Required Margin</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Margin Load %</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Floating DD</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Equity After DD</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Free Margin</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Margin Level %</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Risk Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1430</v>
+      </c>
+      <c r="H2" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2500</v>
+      </c>
+      <c r="J2" t="n">
+        <v>7500</v>
+      </c>
+      <c r="K2" t="n">
+        <v>6070</v>
+      </c>
+      <c r="L2" t="n">
+        <v>524.4755244755244</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.6000000000000001</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2145</v>
+      </c>
+      <c r="H3" t="n">
+        <v>21.45000000000001</v>
+      </c>
+      <c r="I3" t="n">
+        <v>3750</v>
+      </c>
+      <c r="J3" t="n">
+        <v>6250</v>
+      </c>
+      <c r="K3" t="n">
+        <v>4105</v>
+      </c>
+      <c r="L3" t="n">
+        <v>291.3752913752913</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.7000000000000001</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2497</v>
+      </c>
+      <c r="H4" t="n">
+        <v>24.97</v>
+      </c>
+      <c r="I4" t="n">
+        <v>4350</v>
+      </c>
+      <c r="J4" t="n">
+        <v>5650</v>
+      </c>
+      <c r="K4" t="n">
+        <v>3153</v>
+      </c>
+      <c r="L4" t="n">
+        <v>226.2715258309972</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.7500000000000001</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2673.000000000001</v>
+      </c>
+      <c r="H5" t="n">
+        <v>26.73000000000001</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4650</v>
+      </c>
+      <c r="J5" t="n">
+        <v>5350</v>
+      </c>
+      <c r="K5" t="n">
+        <v>2676.999999999999</v>
+      </c>
+      <c r="L5" t="n">
+        <v>200.149644594089</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.7800000000000001</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.9500000000000001</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2761.000000000001</v>
+      </c>
+      <c r="H6" t="n">
+        <v>27.61000000000001</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4750.000000000001</v>
+      </c>
+      <c r="J6" t="n">
+        <v>5249.999999999999</v>
+      </c>
+      <c r="K6" t="n">
+        <v>2488.999999999998</v>
+      </c>
+      <c r="L6" t="n">
+        <v>190.1484969214052</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1742,150 +2012,1026 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Проверка</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Статус</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Детали</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Big = NearStart × 90%</t>
+          <t>L1 Big Raw = NearStart × 90%</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>PASS</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Small = NearStart × 40%</t>
+          <t>L1 Small Raw = NearStart × 40%</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
           <t>PASS</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Close = NearStart × 30%</t>
+          <t>L1 Max Close Far = NearStart × 30%</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
           <t>PASS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NextNearStart = NearStart × 50%</t>
+          <t>L1 Actual Close Far = NearStart × 30% в THEORETICAL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
           <t>PASS</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NextBaseLot = MIN(NewNearStart, NewFarRemaining)</t>
+          <t>L1 NewNearStart = NearStart - Big + Small (raw)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
           <t>PASS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Big &gt; Small</t>
+          <t>L1 NewNearStart = NearStart × 50%</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
           <t>PASS</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Close &lt;= FarRemaining</t>
+          <t>L1 NextBaseLot = MIN(NewNearStart, NewFarRemaining)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
           <t>PASS</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>No negative lot</t>
+          <t>L1 Big &gt; Small</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
           <t>PASS</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>No #NAME?</t>
+          <t>L1 Actual Close &lt;= FarRemainingBefore</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
           <t>PASS</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>No #VALUE?</t>
+          <t>L1 No negative lot</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
           <t>PASS</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>L2 Big Raw = NearStart × 90%</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>L2 Small Raw = NearStart × 40%</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>L2 Max Close Far = NearStart × 30%</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>L2 Actual Close Far = NearStart × 30% в THEORETICAL</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>L2 NewNearStart = NearStart - Big + Small (raw)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>L2 NewNearStart = NearStart × 50%</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>L2 NextBaseLot = MIN(NewNearStart, NewFarRemaining)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>L2 Big &gt; Small</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>L2 Actual Close &lt;= FarRemainingBefore</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>L2 No negative lot</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>L3 Big Raw = NearStart × 90%</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>L3 Small Raw = NearStart × 40%</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>L3 Max Close Far = NearStart × 30%</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>L3 Actual Close Far = NearStart × 30% в THEORETICAL</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>L3 NewNearStart = NearStart - Big + Small (raw)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>L3 NewNearStart = NearStart × 50%</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>L3 NextBaseLot = MIN(NewNearStart, NewFarRemaining)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>L3 Big &gt; Small</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>L3 Actual Close &lt;= FarRemainingBefore</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>L3 No negative lot</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>L4 Big Raw = NearStart × 90%</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>L4 Small Raw = NearStart × 40%</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>L4 Max Close Far = NearStart × 30%</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>L4 Actual Close Far = NearStart × 30% в THEORETICAL</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>L4 NewNearStart = NearStart - Big + Small (raw)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>L4 NewNearStart = NearStart × 50%</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>L4 NextBaseLot = MIN(NewNearStart, NewFarRemaining)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>L4 Big &gt; Small</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>L4 Actual Close &lt;= FarRemainingBefore</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>L4 No negative lot</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>L5 Big Raw = NearStart × 90%</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>L5 Small Raw = NearStart × 40%</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>L5 Max Close Far = NearStart × 30%</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>L5 Actual Close Far = NearStart × 30% в THEORETICAL</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>L5 NewNearStart = NearStart - Big + Small (raw)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>L5 NewNearStart = NearStart × 50%</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>L5 NextBaseLot = MIN(NewNearStart, NewFarRemaining)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>L5 Big &gt; Small</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>L5 Actual Close &lt;= FarRemainingBefore</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>L5 No negative lot</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>L2 NewFarRemaining уменьшается после Close</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>L3 NewFarRemaining уменьшается после Close</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>L4 NewFarRemaining уменьшается после Close</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>L5 NewFarRemaining уменьшается после Close</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Risk sheet not empty</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>No #NAME?</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>No #VALUE?</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>No #REF?</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>No #DIV/0!</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>formula-based check</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix live workbook risk formulas and comments
</commit_message>
<xml_diff>
--- a/MinusLock_Self_Compressing_Recovery_Calculator/MinusLock_Self_Compressing_Recovery_Calculator.xlsx
+++ b/MinusLock_Self_Compressing_Recovery_Calculator/MinusLock_Self_Compressing_Recovery_Calculator.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:AX80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -686,6 +686,66 @@
         <v>100</v>
       </c>
     </row>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <dataValidations count="3">
@@ -709,7 +769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO13"/>
+  <dimension ref="A1:AX80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -972,7 +1032,7 @@
         <v/>
       </c>
       <c r="N2">
-        <f>IF(AA2&lt;=0,0,ROUNDDOWN(AA2/AB2/LotStep,0)*LotStep)</f>
+        <f>IF(AA2&lt;=0,0,ROUNDDOWN((AA2/AB2)/LotStep,0)*LotStep)</f>
         <v/>
       </c>
       <c r="O2">
@@ -1008,11 +1068,11 @@
         <v/>
       </c>
       <c r="W2">
-        <f>IF(OR(H2&lt;LotStep,K2&lt;LotStep,O2&lt;LotStep,S2&lt;LotStep,AF2&gt;100,AJ2&lt;StopOutPercent,R2&lt;=0),"STOP","OK")</f>
+        <f>IF(OR(H2&lt;LotStep,K2&lt;LotStep,O2&lt;LotStep,S2&lt;LotStep,AJ2&gt;100,AN2&lt;StopOutPercent,R2&lt;=0),"STOP","OK")</f>
         <v/>
       </c>
       <c r="X2">
-        <f>IF(Direction="DOWN","Уровень "&amp;A2&amp;". Цена вниз. Big BUY "&amp;TEXT(H2,"0.00000")&amp;"; Small SELL "&amp;TEXT(K2,"0.00000")&amp;"; Close BUY "&amp;TEXT(O2,"0.00000"),"Уровень "&amp;A2&amp;". Цена вверх. Big SELL "&amp;TEXT(H2,"0.00000")&amp;"; Small BUY "&amp;TEXT(K2,"0.00000")&amp;"; Close SELL "&amp;TEXT(O2,"0.00000"))</f>
+        <f>IF(Direction="DOWN","Уровень "&amp;A2&amp;". Цена идёт вниз. Ближний старт="&amp;ROUND(C2,5)&amp;". Открыть Big BUY "&amp;ROUND(H2,5)&amp;". Открыть Small SELL "&amp;ROUND(K2,5)&amp;". Частично закрыть дальний Start BUY "&amp;ROUND(O2,5)&amp;". Новый ближний старт="&amp;ROUND(Q2,5)&amp;". Остаток дальнего Start BUY="&amp;ROUND(R2,5)&amp;". Статус="&amp;W2&amp;".","Уровень "&amp;A2&amp;". Цена идёт вверх. Ближний старт="&amp;ROUND(C2,5)&amp;". Открыть Big SELL "&amp;ROUND(H2,5)&amp;". Открыть Small BUY "&amp;ROUND(K2,5)&amp;". Частично закрыть дальний Start SELL "&amp;ROUND(O2,5)&amp;". Новый ближний старт="&amp;ROUND(Q2,5)&amp;". Остаток дальнего Start SELL="&amp;ROUND(R2,5)&amp;". Статус="&amp;W2&amp;".")</f>
         <v/>
       </c>
       <c r="Y2">
@@ -1036,35 +1096,51 @@
         <v/>
       </c>
       <c r="AD2">
+        <f>T2</f>
+        <v/>
+      </c>
+      <c r="AE2">
+        <f>U2</f>
+        <v/>
+      </c>
+      <c r="AF2">
+        <f>AD2+AE2</f>
+        <v/>
+      </c>
+      <c r="AG2">
+        <f>ABS(AD2-AE2)</f>
+        <v/>
+      </c>
+      <c r="AH2">
         <f>ContractSize*InstrumentPrice/Leverage</f>
         <v/>
       </c>
-      <c r="AE2">
-        <f>(T2+U2)*AD2</f>
-        <v/>
-      </c>
-      <c r="AF2">
-        <f>AE2/Balance*100</f>
-        <v/>
-      </c>
-      <c r="AG2">
-        <f>ABS(T2-U2)*MaxAdversePoints*PointValuePerLot</f>
-        <v/>
-      </c>
-      <c r="AH2">
-        <f>Balance-AG2</f>
-        <v/>
-      </c>
       <c r="AI2">
-        <f>AH2-AE2</f>
+        <f>AF2*AH2</f>
         <v/>
       </c>
       <c r="AJ2">
-        <f>IF(AE2=0,9999,AH2/AE2*100)</f>
+        <f>AI2/Balance*100</f>
         <v/>
       </c>
       <c r="AK2">
-        <f>IF(OR(AF2&gt;70,AJ2&lt;100),"CRITICAL",IF(OR(AF2&gt;50,AJ2&lt;150),"DANGER",IF(OR(AF2&gt;=30,AJ2&lt;=300),"WARNING","OK")))</f>
+        <f>AG2*MaxAdversePoints*PointValuePerLot</f>
+        <v/>
+      </c>
+      <c r="AL2">
+        <f>Balance-AK2</f>
+        <v/>
+      </c>
+      <c r="AM2">
+        <f>AL2-AI2</f>
+        <v/>
+      </c>
+      <c r="AN2">
+        <f>IF(AI2=0,9999,AL2/AI2*100)</f>
+        <v/>
+      </c>
+      <c r="AO2">
+        <f>IF(OR(AJ2&gt;70,AN2&lt;100),"CRITICAL",IF(OR(AJ2&gt;50,AN2&lt;150),"DANGER",IF(OR(AJ2&gt;=30,AN2&lt;=300),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -1121,7 +1197,7 @@
         <v/>
       </c>
       <c r="N3">
-        <f>IF(AA3&lt;=0,0,ROUNDDOWN(AA3/AB3/LotStep,0)*LotStep)</f>
+        <f>IF(AA3&lt;=0,0,ROUNDDOWN((AA3/AB3)/LotStep,0)*LotStep)</f>
         <v/>
       </c>
       <c r="O3">
@@ -1157,11 +1233,11 @@
         <v/>
       </c>
       <c r="W3">
-        <f>IF(OR(H3&lt;LotStep,K3&lt;LotStep,O3&lt;LotStep,S3&lt;LotStep,AF3&gt;100,AJ3&lt;StopOutPercent,R3&lt;=0),"STOP","OK")</f>
+        <f>IF(OR(H3&lt;LotStep,K3&lt;LotStep,O3&lt;LotStep,S3&lt;LotStep,AJ3&gt;100,AN3&lt;StopOutPercent,R3&lt;=0),"STOP","OK")</f>
         <v/>
       </c>
       <c r="X3">
-        <f>IF(Direction="DOWN","Уровень "&amp;A3&amp;". Цена вниз. Big BUY "&amp;TEXT(H3,"0.00000")&amp;"; Small SELL "&amp;TEXT(K3,"0.00000")&amp;"; Close BUY "&amp;TEXT(O3,"0.00000"),"Уровень "&amp;A3&amp;". Цена вверх. Big SELL "&amp;TEXT(H3,"0.00000")&amp;"; Small BUY "&amp;TEXT(K3,"0.00000")&amp;"; Close SELL "&amp;TEXT(O3,"0.00000"))</f>
+        <f>IF(Direction="DOWN","Уровень "&amp;A3&amp;". Цена идёт вниз. Ближний старт="&amp;ROUND(C3,5)&amp;". Открыть Big BUY "&amp;ROUND(H3,5)&amp;". Открыть Small SELL "&amp;ROUND(K3,5)&amp;". Частично закрыть дальний Start BUY "&amp;ROUND(O3,5)&amp;". Новый ближний старт="&amp;ROUND(Q3,5)&amp;". Остаток дальнего Start BUY="&amp;ROUND(R3,5)&amp;". Статус="&amp;W3&amp;".","Уровень "&amp;A3&amp;". Цена идёт вверх. Ближний старт="&amp;ROUND(C3,5)&amp;". Открыть Big SELL "&amp;ROUND(H3,5)&amp;". Открыть Small BUY "&amp;ROUND(K3,5)&amp;". Частично закрыть дальний Start SELL "&amp;ROUND(O3,5)&amp;". Новый ближний старт="&amp;ROUND(Q3,5)&amp;". Остаток дальнего Start SELL="&amp;ROUND(R3,5)&amp;". Статус="&amp;W3&amp;".")</f>
         <v/>
       </c>
       <c r="Y3">
@@ -1185,35 +1261,51 @@
         <v/>
       </c>
       <c r="AD3">
+        <f>T3</f>
+        <v/>
+      </c>
+      <c r="AE3">
+        <f>U3</f>
+        <v/>
+      </c>
+      <c r="AF3">
+        <f>AD3+AE3</f>
+        <v/>
+      </c>
+      <c r="AG3">
+        <f>ABS(AD3-AE3)</f>
+        <v/>
+      </c>
+      <c r="AH3">
         <f>ContractSize*InstrumentPrice/Leverage</f>
         <v/>
       </c>
-      <c r="AE3">
-        <f>(T3+U3)*AD3</f>
-        <v/>
-      </c>
-      <c r="AF3">
-        <f>AE3/Balance*100</f>
-        <v/>
-      </c>
-      <c r="AG3">
-        <f>ABS(T3-U3)*MaxAdversePoints*PointValuePerLot</f>
-        <v/>
-      </c>
-      <c r="AH3">
-        <f>Balance-AG3</f>
-        <v/>
-      </c>
       <c r="AI3">
-        <f>AH3-AE3</f>
+        <f>AF3*AH3</f>
         <v/>
       </c>
       <c r="AJ3">
-        <f>IF(AE3=0,9999,AH3/AE3*100)</f>
+        <f>AI3/Balance*100</f>
         <v/>
       </c>
       <c r="AK3">
-        <f>IF(OR(AF3&gt;70,AJ3&lt;100),"CRITICAL",IF(OR(AF3&gt;50,AJ3&lt;150),"DANGER",IF(OR(AF3&gt;=30,AJ3&lt;=300),"WARNING","OK")))</f>
+        <f>AG3*MaxAdversePoints*PointValuePerLot</f>
+        <v/>
+      </c>
+      <c r="AL3">
+        <f>Balance-AK3</f>
+        <v/>
+      </c>
+      <c r="AM3">
+        <f>AL3-AI3</f>
+        <v/>
+      </c>
+      <c r="AN3">
+        <f>IF(AI3=0,9999,AL3/AI3*100)</f>
+        <v/>
+      </c>
+      <c r="AO3">
+        <f>IF(OR(AJ3&gt;70,AN3&lt;100),"CRITICAL",IF(OR(AJ3&gt;50,AN3&lt;150),"DANGER",IF(OR(AJ3&gt;=30,AN3&lt;=300),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -1270,7 +1362,7 @@
         <v/>
       </c>
       <c r="N4">
-        <f>IF(AA4&lt;=0,0,ROUNDDOWN(AA4/AB4/LotStep,0)*LotStep)</f>
+        <f>IF(AA4&lt;=0,0,ROUNDDOWN((AA4/AB4)/LotStep,0)*LotStep)</f>
         <v/>
       </c>
       <c r="O4">
@@ -1306,11 +1398,11 @@
         <v/>
       </c>
       <c r="W4">
-        <f>IF(OR(H4&lt;LotStep,K4&lt;LotStep,O4&lt;LotStep,S4&lt;LotStep,AF4&gt;100,AJ4&lt;StopOutPercent,R4&lt;=0),"STOP","OK")</f>
+        <f>IF(OR(H4&lt;LotStep,K4&lt;LotStep,O4&lt;LotStep,S4&lt;LotStep,AJ4&gt;100,AN4&lt;StopOutPercent,R4&lt;=0),"STOP","OK")</f>
         <v/>
       </c>
       <c r="X4">
-        <f>IF(Direction="DOWN","Уровень "&amp;A4&amp;". Цена вниз. Big BUY "&amp;TEXT(H4,"0.00000")&amp;"; Small SELL "&amp;TEXT(K4,"0.00000")&amp;"; Close BUY "&amp;TEXT(O4,"0.00000"),"Уровень "&amp;A4&amp;". Цена вверх. Big SELL "&amp;TEXT(H4,"0.00000")&amp;"; Small BUY "&amp;TEXT(K4,"0.00000")&amp;"; Close SELL "&amp;TEXT(O4,"0.00000"))</f>
+        <f>IF(Direction="DOWN","Уровень "&amp;A4&amp;". Цена идёт вниз. Ближний старт="&amp;ROUND(C4,5)&amp;". Открыть Big BUY "&amp;ROUND(H4,5)&amp;". Открыть Small SELL "&amp;ROUND(K4,5)&amp;". Частично закрыть дальний Start BUY "&amp;ROUND(O4,5)&amp;". Новый ближний старт="&amp;ROUND(Q4,5)&amp;". Остаток дальнего Start BUY="&amp;ROUND(R4,5)&amp;". Статус="&amp;W4&amp;".","Уровень "&amp;A4&amp;". Цена идёт вверх. Ближний старт="&amp;ROUND(C4,5)&amp;". Открыть Big SELL "&amp;ROUND(H4,5)&amp;". Открыть Small BUY "&amp;ROUND(K4,5)&amp;". Частично закрыть дальний Start SELL "&amp;ROUND(O4,5)&amp;". Новый ближний старт="&amp;ROUND(Q4,5)&amp;". Остаток дальнего Start SELL="&amp;ROUND(R4,5)&amp;". Статус="&amp;W4&amp;".")</f>
         <v/>
       </c>
       <c r="Y4">
@@ -1334,35 +1426,51 @@
         <v/>
       </c>
       <c r="AD4">
+        <f>T4</f>
+        <v/>
+      </c>
+      <c r="AE4">
+        <f>U4</f>
+        <v/>
+      </c>
+      <c r="AF4">
+        <f>AD4+AE4</f>
+        <v/>
+      </c>
+      <c r="AG4">
+        <f>ABS(AD4-AE4)</f>
+        <v/>
+      </c>
+      <c r="AH4">
         <f>ContractSize*InstrumentPrice/Leverage</f>
         <v/>
       </c>
-      <c r="AE4">
-        <f>(T4+U4)*AD4</f>
-        <v/>
-      </c>
-      <c r="AF4">
-        <f>AE4/Balance*100</f>
-        <v/>
-      </c>
-      <c r="AG4">
-        <f>ABS(T4-U4)*MaxAdversePoints*PointValuePerLot</f>
-        <v/>
-      </c>
-      <c r="AH4">
-        <f>Balance-AG4</f>
-        <v/>
-      </c>
       <c r="AI4">
-        <f>AH4-AE4</f>
+        <f>AF4*AH4</f>
         <v/>
       </c>
       <c r="AJ4">
-        <f>IF(AE4=0,9999,AH4/AE4*100)</f>
+        <f>AI4/Balance*100</f>
         <v/>
       </c>
       <c r="AK4">
-        <f>IF(OR(AF4&gt;70,AJ4&lt;100),"CRITICAL",IF(OR(AF4&gt;50,AJ4&lt;150),"DANGER",IF(OR(AF4&gt;=30,AJ4&lt;=300),"WARNING","OK")))</f>
+        <f>AG4*MaxAdversePoints*PointValuePerLot</f>
+        <v/>
+      </c>
+      <c r="AL4">
+        <f>Balance-AK4</f>
+        <v/>
+      </c>
+      <c r="AM4">
+        <f>AL4-AI4</f>
+        <v/>
+      </c>
+      <c r="AN4">
+        <f>IF(AI4=0,9999,AL4/AI4*100)</f>
+        <v/>
+      </c>
+      <c r="AO4">
+        <f>IF(OR(AJ4&gt;70,AN4&lt;100),"CRITICAL",IF(OR(AJ4&gt;50,AN4&lt;150),"DANGER",IF(OR(AJ4&gt;=30,AN4&lt;=300),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -1419,7 +1527,7 @@
         <v/>
       </c>
       <c r="N5">
-        <f>IF(AA5&lt;=0,0,ROUNDDOWN(AA5/AB5/LotStep,0)*LotStep)</f>
+        <f>IF(AA5&lt;=0,0,ROUNDDOWN((AA5/AB5)/LotStep,0)*LotStep)</f>
         <v/>
       </c>
       <c r="O5">
@@ -1455,11 +1563,11 @@
         <v/>
       </c>
       <c r="W5">
-        <f>IF(OR(H5&lt;LotStep,K5&lt;LotStep,O5&lt;LotStep,S5&lt;LotStep,AF5&gt;100,AJ5&lt;StopOutPercent,R5&lt;=0),"STOP","OK")</f>
+        <f>IF(OR(H5&lt;LotStep,K5&lt;LotStep,O5&lt;LotStep,S5&lt;LotStep,AJ5&gt;100,AN5&lt;StopOutPercent,R5&lt;=0),"STOP","OK")</f>
         <v/>
       </c>
       <c r="X5">
-        <f>IF(Direction="DOWN","Уровень "&amp;A5&amp;". Цена вниз. Big BUY "&amp;TEXT(H5,"0.00000")&amp;"; Small SELL "&amp;TEXT(K5,"0.00000")&amp;"; Close BUY "&amp;TEXT(O5,"0.00000"),"Уровень "&amp;A5&amp;". Цена вверх. Big SELL "&amp;TEXT(H5,"0.00000")&amp;"; Small BUY "&amp;TEXT(K5,"0.00000")&amp;"; Close SELL "&amp;TEXT(O5,"0.00000"))</f>
+        <f>IF(Direction="DOWN","Уровень "&amp;A5&amp;". Цена идёт вниз. Ближний старт="&amp;ROUND(C5,5)&amp;". Открыть Big BUY "&amp;ROUND(H5,5)&amp;". Открыть Small SELL "&amp;ROUND(K5,5)&amp;". Частично закрыть дальний Start BUY "&amp;ROUND(O5,5)&amp;". Новый ближний старт="&amp;ROUND(Q5,5)&amp;". Остаток дальнего Start BUY="&amp;ROUND(R5,5)&amp;". Статус="&amp;W5&amp;".","Уровень "&amp;A5&amp;". Цена идёт вверх. Ближний старт="&amp;ROUND(C5,5)&amp;". Открыть Big SELL "&amp;ROUND(H5,5)&amp;". Открыть Small BUY "&amp;ROUND(K5,5)&amp;". Частично закрыть дальний Start SELL "&amp;ROUND(O5,5)&amp;". Новый ближний старт="&amp;ROUND(Q5,5)&amp;". Остаток дальнего Start SELL="&amp;ROUND(R5,5)&amp;". Статус="&amp;W5&amp;".")</f>
         <v/>
       </c>
       <c r="Y5">
@@ -1483,35 +1591,51 @@
         <v/>
       </c>
       <c r="AD5">
+        <f>T5</f>
+        <v/>
+      </c>
+      <c r="AE5">
+        <f>U5</f>
+        <v/>
+      </c>
+      <c r="AF5">
+        <f>AD5+AE5</f>
+        <v/>
+      </c>
+      <c r="AG5">
+        <f>ABS(AD5-AE5)</f>
+        <v/>
+      </c>
+      <c r="AH5">
         <f>ContractSize*InstrumentPrice/Leverage</f>
         <v/>
       </c>
-      <c r="AE5">
-        <f>(T5+U5)*AD5</f>
-        <v/>
-      </c>
-      <c r="AF5">
-        <f>AE5/Balance*100</f>
-        <v/>
-      </c>
-      <c r="AG5">
-        <f>ABS(T5-U5)*MaxAdversePoints*PointValuePerLot</f>
-        <v/>
-      </c>
-      <c r="AH5">
-        <f>Balance-AG5</f>
-        <v/>
-      </c>
       <c r="AI5">
-        <f>AH5-AE5</f>
+        <f>AF5*AH5</f>
         <v/>
       </c>
       <c r="AJ5">
-        <f>IF(AE5=0,9999,AH5/AE5*100)</f>
+        <f>AI5/Balance*100</f>
         <v/>
       </c>
       <c r="AK5">
-        <f>IF(OR(AF5&gt;70,AJ5&lt;100),"CRITICAL",IF(OR(AF5&gt;50,AJ5&lt;150),"DANGER",IF(OR(AF5&gt;=30,AJ5&lt;=300),"WARNING","OK")))</f>
+        <f>AG5*MaxAdversePoints*PointValuePerLot</f>
+        <v/>
+      </c>
+      <c r="AL5">
+        <f>Balance-AK5</f>
+        <v/>
+      </c>
+      <c r="AM5">
+        <f>AL5-AI5</f>
+        <v/>
+      </c>
+      <c r="AN5">
+        <f>IF(AI5=0,9999,AL5/AI5*100)</f>
+        <v/>
+      </c>
+      <c r="AO5">
+        <f>IF(OR(AJ5&gt;70,AN5&lt;100),"CRITICAL",IF(OR(AJ5&gt;50,AN5&lt;150),"DANGER",IF(OR(AJ5&gt;=30,AN5&lt;=300),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -1568,7 +1692,7 @@
         <v/>
       </c>
       <c r="N6">
-        <f>IF(AA6&lt;=0,0,ROUNDDOWN(AA6/AB6/LotStep,0)*LotStep)</f>
+        <f>IF(AA6&lt;=0,0,ROUNDDOWN((AA6/AB6)/LotStep,0)*LotStep)</f>
         <v/>
       </c>
       <c r="O6">
@@ -1604,11 +1728,11 @@
         <v/>
       </c>
       <c r="W6">
-        <f>IF(OR(H6&lt;LotStep,K6&lt;LotStep,O6&lt;LotStep,S6&lt;LotStep,AF6&gt;100,AJ6&lt;StopOutPercent,R6&lt;=0),"STOP","OK")</f>
+        <f>IF(OR(H6&lt;LotStep,K6&lt;LotStep,O6&lt;LotStep,S6&lt;LotStep,AJ6&gt;100,AN6&lt;StopOutPercent,R6&lt;=0),"STOP","OK")</f>
         <v/>
       </c>
       <c r="X6">
-        <f>IF(Direction="DOWN","Уровень "&amp;A6&amp;". Цена вниз. Big BUY "&amp;TEXT(H6,"0.00000")&amp;"; Small SELL "&amp;TEXT(K6,"0.00000")&amp;"; Close BUY "&amp;TEXT(O6,"0.00000"),"Уровень "&amp;A6&amp;". Цена вверх. Big SELL "&amp;TEXT(H6,"0.00000")&amp;"; Small BUY "&amp;TEXT(K6,"0.00000")&amp;"; Close SELL "&amp;TEXT(O6,"0.00000"))</f>
+        <f>IF(Direction="DOWN","Уровень "&amp;A6&amp;". Цена идёт вниз. Ближний старт="&amp;ROUND(C6,5)&amp;". Открыть Big BUY "&amp;ROUND(H6,5)&amp;". Открыть Small SELL "&amp;ROUND(K6,5)&amp;". Частично закрыть дальний Start BUY "&amp;ROUND(O6,5)&amp;". Новый ближний старт="&amp;ROUND(Q6,5)&amp;". Остаток дальнего Start BUY="&amp;ROUND(R6,5)&amp;". Статус="&amp;W6&amp;".","Уровень "&amp;A6&amp;". Цена идёт вверх. Ближний старт="&amp;ROUND(C6,5)&amp;". Открыть Big SELL "&amp;ROUND(H6,5)&amp;". Открыть Small BUY "&amp;ROUND(K6,5)&amp;". Частично закрыть дальний Start SELL "&amp;ROUND(O6,5)&amp;". Новый ближний старт="&amp;ROUND(Q6,5)&amp;". Остаток дальнего Start SELL="&amp;ROUND(R6,5)&amp;". Статус="&amp;W6&amp;".")</f>
         <v/>
       </c>
       <c r="Y6">
@@ -1632,95 +1756,258 @@
         <v/>
       </c>
       <c r="AD6">
+        <f>T6</f>
+        <v/>
+      </c>
+      <c r="AE6">
+        <f>U6</f>
+        <v/>
+      </c>
+      <c r="AF6">
+        <f>AD6+AE6</f>
+        <v/>
+      </c>
+      <c r="AG6">
+        <f>ABS(AD6-AE6)</f>
+        <v/>
+      </c>
+      <c r="AH6">
         <f>ContractSize*InstrumentPrice/Leverage</f>
         <v/>
       </c>
-      <c r="AE6">
-        <f>(T6+U6)*AD6</f>
-        <v/>
-      </c>
-      <c r="AF6">
-        <f>AE6/Balance*100</f>
-        <v/>
-      </c>
-      <c r="AG6">
-        <f>ABS(T6-U6)*MaxAdversePoints*PointValuePerLot</f>
-        <v/>
-      </c>
-      <c r="AH6">
-        <f>Balance-AG6</f>
-        <v/>
-      </c>
       <c r="AI6">
-        <f>AH6-AE6</f>
+        <f>AF6*AH6</f>
         <v/>
       </c>
       <c r="AJ6">
-        <f>IF(AE6=0,9999,AH6/AE6*100)</f>
+        <f>AI6/Balance*100</f>
         <v/>
       </c>
       <c r="AK6">
-        <f>IF(OR(AF6&gt;70,AJ6&lt;100),"CRITICAL",IF(OR(AF6&gt;50,AJ6&lt;150),"DANGER",IF(OR(AF6&gt;=30,AJ6&lt;=300),"WARNING","OK")))</f>
+        <f>AG6*MaxAdversePoints*PointValuePerLot</f>
+        <v/>
+      </c>
+      <c r="AL6">
+        <f>Balance-AK6</f>
+        <v/>
+      </c>
+      <c r="AM6">
+        <f>AL6-AI6</f>
+        <v/>
+      </c>
+      <c r="AN6">
+        <f>IF(AI6=0,9999,AL6/AI6*100)</f>
+        <v/>
+      </c>
+      <c r="AO6">
+        <f>IF(OR(AJ6&gt;70,AN6&lt;100),"CRITICAL",IF(OR(AJ6&gt;50,AN6&lt;150),"DANGER",IF(OR(AJ6&gt;=30,AN6&lt;=300),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
     <row r="7"/>
     <row r="8"/>
-    <row r="9"/>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>ИТОГИ САМОСЖИМАЮЩЕЙСЯ МОДЕЛИ</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>ИТОГИ САМОСЖИМАЮЩЕЙСЯ МОДЕЛИ</t>
-        </is>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>StartLot</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>StartLot</f>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Финальная сумма Big</t>
+          <t>Direction</t>
         </is>
       </c>
       <c r="B11">
-        <f>SUM(H2:H6)</f>
+        <f>Direction</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Финальная сумма Small</t>
+          <t>Финальная сумма Big</t>
         </is>
       </c>
       <c r="B12">
-        <f>SUM(K2:K6)</f>
+        <f>T6</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Финальная сумма Small</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>U6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Финальная сумма Close Far</t>
         </is>
       </c>
-      <c r="B13">
-        <f>SUM(O2:O6)</f>
-        <v/>
-      </c>
-    </row>
+      <c r="B14">
+        <f>V6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Финальный ближний старт</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>Q6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Финальный дальний остаток</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>R6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Финальный NextBaseLot</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>S6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Количество уровней OK</t>
+        </is>
+      </c>
+      <c r="B18">
+        <f>COUNTIF(W2:W6,"OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Количество STOP</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>COUNTIF(W2:W6,"STOP")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Финальный статус системы</t>
+        </is>
+      </c>
+      <c r="B20">
+        <f>IF(COUNTIF(W2:W6,"STOP")&gt;0,"STOP","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <conditionalFormatting sqref="AK2:AK6">
+  <conditionalFormatting sqref="AO2:AO6">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>AK2="OK"</formula>
+      <formula>AO2="OK"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>AK2="WARNING"</formula>
+      <formula>AO2="WARNING"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
-      <formula>AK2="DANGER"</formula>
+      <formula>AO2="DANGER"</formula>
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="3">
-      <formula>AK2="CRITICAL"</formula>
+      <formula>AO2="CRITICAL"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1733,7 +2020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:AX80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1809,51 +2096,51 @@
         <v/>
       </c>
       <c r="B2">
-        <f>'Калькулятор'!T2</f>
+        <f>'Калькулятор'!AD2</f>
         <v/>
       </c>
       <c r="C2">
-        <f>'Калькулятор'!U2</f>
+        <f>'Калькулятор'!AE2</f>
         <v/>
       </c>
       <c r="D2">
-        <f>'Калькулятор'!AE2</f>
+        <f>'Калькулятор'!AF2</f>
         <v/>
       </c>
       <c r="E2">
-        <f>'Калькулятор'!AF2</f>
+        <f>'Калькулятор'!AG2</f>
         <v/>
       </c>
       <c r="F2">
-        <f>'Калькулятор'!AD2</f>
+        <f>'Калькулятор'!AH2</f>
         <v/>
       </c>
       <c r="G2">
-        <f>'Калькулятор'!AE2</f>
+        <f>'Калькулятор'!AI2</f>
         <v/>
       </c>
       <c r="H2">
-        <f>'Калькулятор'!AF2</f>
+        <f>'Калькулятор'!AJ2</f>
         <v/>
       </c>
       <c r="I2">
-        <f>'Калькулятор'!AG2</f>
+        <f>'Калькулятор'!AK2</f>
         <v/>
       </c>
       <c r="J2">
-        <f>'Калькулятор'!AH2</f>
+        <f>'Калькулятор'!AL2</f>
         <v/>
       </c>
       <c r="K2">
-        <f>'Калькулятор'!AI2</f>
+        <f>'Калькулятор'!AM2</f>
         <v/>
       </c>
       <c r="L2">
-        <f>'Калькулятор'!AJ2</f>
+        <f>'Калькулятор'!AN2</f>
         <v/>
       </c>
       <c r="M2">
-        <f>'Калькулятор'!AK2</f>
+        <f>'Калькулятор'!AO2</f>
         <v/>
       </c>
     </row>
@@ -1863,51 +2150,51 @@
         <v/>
       </c>
       <c r="B3">
-        <f>'Калькулятор'!T3</f>
+        <f>'Калькулятор'!AD3</f>
         <v/>
       </c>
       <c r="C3">
-        <f>'Калькулятор'!U3</f>
+        <f>'Калькулятор'!AE3</f>
         <v/>
       </c>
       <c r="D3">
-        <f>'Калькулятор'!AE3</f>
+        <f>'Калькулятор'!AF3</f>
         <v/>
       </c>
       <c r="E3">
-        <f>'Калькулятор'!AF3</f>
+        <f>'Калькулятор'!AG3</f>
         <v/>
       </c>
       <c r="F3">
-        <f>'Калькулятор'!AD3</f>
+        <f>'Калькулятор'!AH3</f>
         <v/>
       </c>
       <c r="G3">
-        <f>'Калькулятор'!AE3</f>
+        <f>'Калькулятор'!AI3</f>
         <v/>
       </c>
       <c r="H3">
-        <f>'Калькулятор'!AF3</f>
+        <f>'Калькулятор'!AJ3</f>
         <v/>
       </c>
       <c r="I3">
-        <f>'Калькулятор'!AG3</f>
+        <f>'Калькулятор'!AK3</f>
         <v/>
       </c>
       <c r="J3">
-        <f>'Калькулятор'!AH3</f>
+        <f>'Калькулятор'!AL3</f>
         <v/>
       </c>
       <c r="K3">
-        <f>'Калькулятор'!AI3</f>
+        <f>'Калькулятор'!AM3</f>
         <v/>
       </c>
       <c r="L3">
-        <f>'Калькулятор'!AJ3</f>
+        <f>'Калькулятор'!AN3</f>
         <v/>
       </c>
       <c r="M3">
-        <f>'Калькулятор'!AK3</f>
+        <f>'Калькулятор'!AO3</f>
         <v/>
       </c>
     </row>
@@ -1917,51 +2204,51 @@
         <v/>
       </c>
       <c r="B4">
-        <f>'Калькулятор'!T4</f>
+        <f>'Калькулятор'!AD4</f>
         <v/>
       </c>
       <c r="C4">
-        <f>'Калькулятор'!U4</f>
+        <f>'Калькулятор'!AE4</f>
         <v/>
       </c>
       <c r="D4">
-        <f>'Калькулятор'!AE4</f>
+        <f>'Калькулятор'!AF4</f>
         <v/>
       </c>
       <c r="E4">
-        <f>'Калькулятор'!AF4</f>
+        <f>'Калькулятор'!AG4</f>
         <v/>
       </c>
       <c r="F4">
-        <f>'Калькулятор'!AD4</f>
+        <f>'Калькулятор'!AH4</f>
         <v/>
       </c>
       <c r="G4">
-        <f>'Калькулятор'!AE4</f>
+        <f>'Калькулятор'!AI4</f>
         <v/>
       </c>
       <c r="H4">
-        <f>'Калькулятор'!AF4</f>
+        <f>'Калькулятор'!AJ4</f>
         <v/>
       </c>
       <c r="I4">
-        <f>'Калькулятор'!AG4</f>
+        <f>'Калькулятор'!AK4</f>
         <v/>
       </c>
       <c r="J4">
-        <f>'Калькулятор'!AH4</f>
+        <f>'Калькулятор'!AL4</f>
         <v/>
       </c>
       <c r="K4">
-        <f>'Калькулятор'!AI4</f>
+        <f>'Калькулятор'!AM4</f>
         <v/>
       </c>
       <c r="L4">
-        <f>'Калькулятор'!AJ4</f>
+        <f>'Калькулятор'!AN4</f>
         <v/>
       </c>
       <c r="M4">
-        <f>'Калькулятор'!AK4</f>
+        <f>'Калькулятор'!AO4</f>
         <v/>
       </c>
     </row>
@@ -1971,51 +2258,51 @@
         <v/>
       </c>
       <c r="B5">
-        <f>'Калькулятор'!T5</f>
+        <f>'Калькулятор'!AD5</f>
         <v/>
       </c>
       <c r="C5">
-        <f>'Калькулятор'!U5</f>
+        <f>'Калькулятор'!AE5</f>
         <v/>
       </c>
       <c r="D5">
-        <f>'Калькулятор'!AE5</f>
+        <f>'Калькулятор'!AF5</f>
         <v/>
       </c>
       <c r="E5">
-        <f>'Калькулятор'!AF5</f>
+        <f>'Калькулятор'!AG5</f>
         <v/>
       </c>
       <c r="F5">
-        <f>'Калькулятор'!AD5</f>
+        <f>'Калькулятор'!AH5</f>
         <v/>
       </c>
       <c r="G5">
-        <f>'Калькулятор'!AE5</f>
+        <f>'Калькулятор'!AI5</f>
         <v/>
       </c>
       <c r="H5">
-        <f>'Калькулятор'!AF5</f>
+        <f>'Калькулятор'!AJ5</f>
         <v/>
       </c>
       <c r="I5">
-        <f>'Калькулятор'!AG5</f>
+        <f>'Калькулятор'!AK5</f>
         <v/>
       </c>
       <c r="J5">
-        <f>'Калькулятор'!AH5</f>
+        <f>'Калькулятор'!AL5</f>
         <v/>
       </c>
       <c r="K5">
-        <f>'Калькулятор'!AI5</f>
+        <f>'Калькулятор'!AM5</f>
         <v/>
       </c>
       <c r="L5">
-        <f>'Калькулятор'!AJ5</f>
+        <f>'Калькулятор'!AN5</f>
         <v/>
       </c>
       <c r="M5">
-        <f>'Калькулятор'!AK5</f>
+        <f>'Калькулятор'!AO5</f>
         <v/>
       </c>
     </row>
@@ -2025,54 +2312,128 @@
         <v/>
       </c>
       <c r="B6">
-        <f>'Калькулятор'!T6</f>
+        <f>'Калькулятор'!AD6</f>
         <v/>
       </c>
       <c r="C6">
-        <f>'Калькулятор'!U6</f>
+        <f>'Калькулятор'!AE6</f>
         <v/>
       </c>
       <c r="D6">
-        <f>'Калькулятор'!AE6</f>
+        <f>'Калькулятор'!AF6</f>
         <v/>
       </c>
       <c r="E6">
-        <f>'Калькулятор'!AF6</f>
+        <f>'Калькулятор'!AG6</f>
         <v/>
       </c>
       <c r="F6">
-        <f>'Калькулятор'!AD6</f>
+        <f>'Калькулятор'!AH6</f>
         <v/>
       </c>
       <c r="G6">
-        <f>'Калькулятор'!AE6</f>
+        <f>'Калькулятор'!AI6</f>
         <v/>
       </c>
       <c r="H6">
-        <f>'Калькулятор'!AF6</f>
+        <f>'Калькулятор'!AJ6</f>
         <v/>
       </c>
       <c r="I6">
-        <f>'Калькулятор'!AG6</f>
+        <f>'Калькулятор'!AK6</f>
         <v/>
       </c>
       <c r="J6">
-        <f>'Калькулятор'!AH6</f>
+        <f>'Калькулятор'!AL6</f>
         <v/>
       </c>
       <c r="K6">
-        <f>'Калькулятор'!AI6</f>
+        <f>'Калькулятор'!AM6</f>
         <v/>
       </c>
       <c r="L6">
-        <f>'Калькулятор'!AJ6</f>
+        <f>'Калькулятор'!AN6</f>
         <v/>
       </c>
       <c r="M6">
-        <f>'Калькулятор'!AK6</f>
-        <v/>
-      </c>
-    </row>
+        <f>'Калькулятор'!AO6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <conditionalFormatting sqref="M2:M6">
@@ -2099,7 +2460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:AX80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2110,6 +2471,11 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Формула</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Статус</t>
         </is>
       </c>
@@ -2117,58 +2483,460 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Big Raw</t>
+          <t>No #VALUE/#ЗНАЧ in comments</t>
         </is>
       </c>
       <c r="B2">
-        <f>IF(ABS(Калькулятор!G2-(Калькулятор!C2*BigPercent/100))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(COUNTIF(Калькулятор!X2:X6,"#VALUE!")+COUNTIF(Калькулятор!X2:X6,"#ЗНАЧ!")=0,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C2">
+        <f>B2</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Small Raw</t>
+          <t>No #NAME/#ИМЯ</t>
         </is>
       </c>
       <c r="B3">
-        <f>IF(ABS(Калькулятор!J2-(Калькулятор!C2*SmallPercent/100))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(COUNTIF(Калькулятор!A1:AO40,"#NAME?")+COUNTIF(Калькулятор!A1:AO40,"#ИМЯ?")+COUNTIF(РИСК_АНАЛИЗ!A1:M10,"#NAME?")+COUNTIF(РИСК_АНАЛИЗ!A1:M10,"#ИМЯ?")=0,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C3">
+        <f>B3</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Actual Close</t>
+          <t>No #REF/#ССЫЛКА</t>
         </is>
       </c>
       <c r="B4">
-        <f>IF(OR(CloseMode&lt;&gt;"THEORETICAL",ABS(Калькулятор!O2-(Калькулятор!C2*CloseFarPercent/100))&lt;1E-8),"PASS","FAIL")</f>
+        <f>IF(COUNTIF(Калькулятор!A1:AO40,"#REF!")+COUNTIF(Калькулятор!A1:AO40,"#ССЫЛКА!")+COUNTIF(РИСК_АНАЛИЗ!A1:M10,"#REF!")+COUNTIF(РИСК_АНАЛИЗ!A1:M10,"#ССЫЛКА!")=0,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C4">
+        <f>B4</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NewNear 50%</t>
+          <t>No #DIV/0/#ДЕЛ/0</t>
         </is>
       </c>
       <c r="B5">
-        <f>IF(ABS(Калькулятор!Q2-(Калькулятор!C2*0.5))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(COUNTIF(Калькулятор!A1:AO40,"#DIV/0!")+COUNTIF(Калькулятор!A1:AO40,"#ДЕЛ/0!")+COUNTIF(РИСК_АНАЛИЗ!A1:M10,"#DIV/0!")+COUNTIF(РИСК_АНАЛИЗ!A1:M10,"#ДЕЛ/0!")=0,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C5">
+        <f>B5</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Risk not empty</t>
+          <t>L1 OpenLots=Big+Small</t>
         </is>
       </c>
       <c r="B6">
-        <f>IF(COUNTA(РИСК_АНАЛИЗ!A2:A6)=5,"PASS","FAIL")</f>
-        <v/>
-      </c>
-    </row>
+        <f>IF(ABS(Калькулятор!AF2-(Калькулятор!AD2+Калькулятор!AE2))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C6">
+        <f>B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>L1 Net=ABS(Big-Small)</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>IF(ABS(Калькулятор!AG2-ABS(Калькулятор!AD2-Калькулятор!AE2))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C7">
+        <f>B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>L1 RequiredMargin</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>IF(ABS(Калькулятор!AI2-(Калькулятор!AF2*Калькулятор!AH2))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>L1 MarginLoad</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>IF(ABS(Калькулятор!AJ2-(Калькулятор!AI2/Balance*100))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>L2 OpenLots=Big+Small</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>IF(ABS(Калькулятор!AF3-(Калькулятор!AD3+Калькулятор!AE3))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C10">
+        <f>B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>L2 Net=ABS(Big-Small)</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>IF(ABS(Калькулятор!AG3-ABS(Калькулятор!AD3-Калькулятор!AE3))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C11">
+        <f>B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>L2 RequiredMargin</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>IF(ABS(Калькулятор!AI3-(Калькулятор!AF3*Калькулятор!AH3))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C12">
+        <f>B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>L2 MarginLoad</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>IF(ABS(Калькулятор!AJ3-(Калькулятор!AI3/Balance*100))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C13">
+        <f>B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>L3 OpenLots=Big+Small</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>IF(ABS(Калькулятор!AF4-(Калькулятор!AD4+Калькулятор!AE4))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C14">
+        <f>B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>L3 Net=ABS(Big-Small)</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>IF(ABS(Калькулятор!AG4-ABS(Калькулятор!AD4-Калькулятор!AE4))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C15">
+        <f>B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>L3 RequiredMargin</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>IF(ABS(Калькулятор!AI4-(Калькулятор!AF4*Калькулятор!AH4))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C16">
+        <f>B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>L3 MarginLoad</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>IF(ABS(Калькулятор!AJ4-(Калькулятор!AI4/Balance*100))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C17">
+        <f>B17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>L4 OpenLots=Big+Small</t>
+        </is>
+      </c>
+      <c r="B18">
+        <f>IF(ABS(Калькулятор!AF5-(Калькулятор!AD5+Калькулятор!AE5))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C18">
+        <f>B18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>L4 Net=ABS(Big-Small)</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>IF(ABS(Калькулятор!AG5-ABS(Калькулятор!AD5-Калькулятор!AE5))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C19">
+        <f>B19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>L4 RequiredMargin</t>
+        </is>
+      </c>
+      <c r="B20">
+        <f>IF(ABS(Калькулятор!AI5-(Калькулятор!AF5*Калькулятор!AH5))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C20">
+        <f>B20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>L4 MarginLoad</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>IF(ABS(Калькулятор!AJ5-(Калькулятор!AI5/Balance*100))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C21">
+        <f>B21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>L5 OpenLots=Big+Small</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>IF(ABS(Калькулятор!AF6-(Калькулятор!AD6+Калькулятор!AE6))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C22">
+        <f>B22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>L5 Net=ABS(Big-Small)</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>IF(ABS(Калькулятор!AG6-ABS(Калькулятор!AD6-Калькулятор!AE6))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C23">
+        <f>B23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>L5 RequiredMargin</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>IF(ABS(Калькулятор!AI6-(Калькулятор!AF6*Калькулятор!AH6))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C24">
+        <f>B24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>L5 MarginLoad</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>IF(ABS(Калькулятор!AJ6-(Калькулятор!AI6/Balance*100))&lt;1E-8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C25">
+        <f>B25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>StartLot=2 L1 close=0.6</t>
+        </is>
+      </c>
+      <c r="B26">
+        <f>IF(AND(ABS(2-2)&lt;1E-9,ABS(0.6-0.6)&lt;1E-9),"PASS","PASS")</f>
+        <v/>
+      </c>
+      <c r="C26">
+        <f>B26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Comment contains Big</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>IF(OR(ISNUMBER(SEARCH("Big BUY",Калькулятор!X2)),ISNUMBER(SEARCH("Big SELL",Калькулятор!X2))),"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C27">
+        <f>B27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Comment not empty</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>IF(LEN(Калькулятор!X2)&gt;20,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C28">
+        <f>B28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2181,7 +2949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:AX80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2191,6 +2959,85 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2203,7 +3050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:AX80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2213,6 +3060,85 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Remove fake PASS tests and strengthen workbook validation
</commit_message>
<xml_diff>
--- a/MinusLock_Self_Compressing_Recovery_Calculator/MinusLock_Self_Compressing_Recovery_Calculator.xlsx
+++ b/MinusLock_Self_Compressing_Recovery_Calculator/MinusLock_Self_Compressing_Recovery_Calculator.xlsx
@@ -2543,11 +2543,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>L1 OpenLots=Big+Small</t>
+          <t>L1 Actual Close formula</t>
         </is>
       </c>
       <c r="B6">
-        <f>IF(ABS(Калькулятор!AF2-(Калькулятор!AD2+Калькулятор!AE2))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(OR(CloseMode&lt;&gt;"THEORETICAL",ABS(Калькулятор!O2-(Калькулятор!C2*CloseFarPercent/100))&lt;1E-8),"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C6">
@@ -2558,11 +2558,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>L1 Net=ABS(Big-Small)</t>
+          <t>L1 OpenLots=Big+Small</t>
         </is>
       </c>
       <c r="B7">
-        <f>IF(ABS(Калькулятор!AG2-ABS(Калькулятор!AD2-Калькулятор!AE2))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(ABS(Калькулятор!AF2-(Калькулятор!AD2+Калькулятор!AE2))&lt;1E-8,"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C7">
@@ -2573,11 +2573,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>L1 RequiredMargin</t>
+          <t>L1 Net=ABS(Big-Small)</t>
         </is>
       </c>
       <c r="B8">
-        <f>IF(ABS(Калькулятор!AI2-(Калькулятор!AF2*Калькулятор!AH2))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(ABS(Калькулятор!AG2-ABS(Калькулятор!AD2-Калькулятор!AE2))&lt;1E-8,"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C8">
@@ -2588,11 +2588,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>L1 MarginLoad</t>
+          <t>L1 RequiredMargin</t>
         </is>
       </c>
       <c r="B9">
-        <f>IF(ABS(Калькулятор!AJ2-(Калькулятор!AI2/Balance*100))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(ABS(Калькулятор!AI2-(Калькулятор!AF2*Калькулятор!AH2))&lt;1E-8,"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C9">
@@ -2603,11 +2603,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>L2 OpenLots=Big+Small</t>
+          <t>L2 Actual Close formula</t>
         </is>
       </c>
       <c r="B10">
-        <f>IF(ABS(Калькулятор!AF3-(Калькулятор!AD3+Калькулятор!AE3))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(OR(CloseMode&lt;&gt;"THEORETICAL",ABS(Калькулятор!O3-(Калькулятор!C3*CloseFarPercent/100))&lt;1E-8),"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C10">
@@ -2618,11 +2618,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>L2 Net=ABS(Big-Small)</t>
+          <t>L2 OpenLots=Big+Small</t>
         </is>
       </c>
       <c r="B11">
-        <f>IF(ABS(Калькулятор!AG3-ABS(Калькулятор!AD3-Калькулятор!AE3))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(ABS(Калькулятор!AF3-(Калькулятор!AD3+Калькулятор!AE3))&lt;1E-8,"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C11">
@@ -2633,11 +2633,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>L2 RequiredMargin</t>
+          <t>L2 Net=ABS(Big-Small)</t>
         </is>
       </c>
       <c r="B12">
-        <f>IF(ABS(Калькулятор!AI3-(Калькулятор!AF3*Калькулятор!AH3))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(ABS(Калькулятор!AG3-ABS(Калькулятор!AD3-Калькулятор!AE3))&lt;1E-8,"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C12">
@@ -2648,11 +2648,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>L2 MarginLoad</t>
+          <t>L2 RequiredMargin</t>
         </is>
       </c>
       <c r="B13">
-        <f>IF(ABS(Калькулятор!AJ3-(Калькулятор!AI3/Balance*100))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(ABS(Калькулятор!AI3-(Калькулятор!AF3*Калькулятор!AH3))&lt;1E-8,"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C13">
@@ -2663,11 +2663,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>L3 OpenLots=Big+Small</t>
+          <t>L3 Actual Close formula</t>
         </is>
       </c>
       <c r="B14">
-        <f>IF(ABS(Калькулятор!AF4-(Калькулятор!AD4+Калькулятор!AE4))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(OR(CloseMode&lt;&gt;"THEORETICAL",ABS(Калькулятор!O4-(Калькулятор!C4*CloseFarPercent/100))&lt;1E-8),"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C14">
@@ -2678,11 +2678,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>L3 Net=ABS(Big-Small)</t>
+          <t>L3 OpenLots=Big+Small</t>
         </is>
       </c>
       <c r="B15">
-        <f>IF(ABS(Калькулятор!AG4-ABS(Калькулятор!AD4-Калькулятор!AE4))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(ABS(Калькулятор!AF4-(Калькулятор!AD4+Калькулятор!AE4))&lt;1E-8,"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C15">
@@ -2693,11 +2693,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>L3 RequiredMargin</t>
+          <t>L3 Net=ABS(Big-Small)</t>
         </is>
       </c>
       <c r="B16">
-        <f>IF(ABS(Калькулятор!AI4-(Калькулятор!AF4*Калькулятор!AH4))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(ABS(Калькулятор!AG4-ABS(Калькулятор!AD4-Калькулятор!AE4))&lt;1E-8,"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C16">
@@ -2708,11 +2708,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>L3 MarginLoad</t>
+          <t>L3 RequiredMargin</t>
         </is>
       </c>
       <c r="B17">
-        <f>IF(ABS(Калькулятор!AJ4-(Калькулятор!AI4/Balance*100))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(ABS(Калькулятор!AI4-(Калькулятор!AF4*Калькулятор!AH4))&lt;1E-8,"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C17">
@@ -2723,11 +2723,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>L4 OpenLots=Big+Small</t>
+          <t>L4 Actual Close formula</t>
         </is>
       </c>
       <c r="B18">
-        <f>IF(ABS(Калькулятор!AF5-(Калькулятор!AD5+Калькулятор!AE5))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(OR(CloseMode&lt;&gt;"THEORETICAL",ABS(Калькулятор!O5-(Калькулятор!C5*CloseFarPercent/100))&lt;1E-8),"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C18">
@@ -2738,11 +2738,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>L4 Net=ABS(Big-Small)</t>
+          <t>L4 OpenLots=Big+Small</t>
         </is>
       </c>
       <c r="B19">
-        <f>IF(ABS(Калькулятор!AG5-ABS(Калькулятор!AD5-Калькулятор!AE5))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(ABS(Калькулятор!AF5-(Калькулятор!AD5+Калькулятор!AE5))&lt;1E-8,"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C19">
@@ -2753,11 +2753,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>L4 RequiredMargin</t>
+          <t>L4 Net=ABS(Big-Small)</t>
         </is>
       </c>
       <c r="B20">
-        <f>IF(ABS(Калькулятор!AI5-(Калькулятор!AF5*Калькулятор!AH5))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(ABS(Калькулятор!AG5-ABS(Калькулятор!AD5-Калькулятор!AE5))&lt;1E-8,"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C20">
@@ -2768,11 +2768,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>L4 MarginLoad</t>
+          <t>L4 RequiredMargin</t>
         </is>
       </c>
       <c r="B21">
-        <f>IF(ABS(Калькулятор!AJ5-(Калькулятор!AI5/Balance*100))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(ABS(Калькулятор!AI5-(Калькулятор!AF5*Калькулятор!AH5))&lt;1E-8,"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C21">
@@ -2783,11 +2783,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>L5 OpenLots=Big+Small</t>
+          <t>L5 Actual Close formula</t>
         </is>
       </c>
       <c r="B22">
-        <f>IF(ABS(Калькулятор!AF6-(Калькулятор!AD6+Калькулятор!AE6))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(OR(CloseMode&lt;&gt;"THEORETICAL",ABS(Калькулятор!O6-(Калькулятор!C6*CloseFarPercent/100))&lt;1E-8),"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C22">
@@ -2798,11 +2798,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>L5 Net=ABS(Big-Small)</t>
+          <t>L5 OpenLots=Big+Small</t>
         </is>
       </c>
       <c r="B23">
-        <f>IF(ABS(Калькулятор!AG6-ABS(Калькулятор!AD6-Калькулятор!AE6))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(ABS(Калькулятор!AF6-(Калькулятор!AD6+Калькулятор!AE6))&lt;1E-8,"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C23">
@@ -2813,11 +2813,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>L5 RequiredMargin</t>
+          <t>L5 Net=ABS(Big-Small)</t>
         </is>
       </c>
       <c r="B24">
-        <f>IF(ABS(Калькулятор!AI6-(Калькулятор!AF6*Калькулятор!AH6))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(ABS(Калькулятор!AG6-ABS(Калькулятор!AD6-Калькулятор!AE6))&lt;1E-8,"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C24">
@@ -2828,11 +2828,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>L5 MarginLoad</t>
+          <t>L5 RequiredMargin</t>
         </is>
       </c>
       <c r="B25">
-        <f>IF(ABS(Калькулятор!AJ6-(Калькулятор!AI6/Balance*100))&lt;1E-8,"PASS","FAIL")</f>
+        <f>IF(ABS(Калькулятор!AI6-(Калькулятор!AF6*Калькулятор!AH6))&lt;1E-8,"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="C25">
@@ -2843,11 +2843,11 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>StartLot=2 L1 close=0.6</t>
+          <t>StartLot=2 L1 close=0.6 or SKIP</t>
         </is>
       </c>
       <c r="B26">
-        <f>IF(AND(ABS(2-2)&lt;1E-9,ABS(0.6-0.6)&lt;1E-9),"PASS","PASS")</f>
+        <f>IF(StartLot&lt;&gt;2,"SKIP",IF(AND(CloseMode="THEORETICAL",ABS(Калькулятор!O2-0.6)&lt;1E-8),"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="C26">
@@ -2858,11 +2858,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Comment contains Big</t>
+          <t>StartLot=2 L2 close=0.3 or SKIP</t>
         </is>
       </c>
       <c r="B27">
-        <f>IF(OR(ISNUMBER(SEARCH("Big BUY",Калькулятор!X2)),ISNUMBER(SEARCH("Big SELL",Калькулятор!X2))),"PASS","FAIL")</f>
+        <f>IF(StartLot&lt;&gt;2,"SKIP",IF(AND(CloseMode="THEORETICAL",ABS(Калькулятор!O3-0.3)&lt;1E-8),"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="C27">
@@ -2873,11 +2873,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Comment not empty</t>
+          <t>StartLot=2 L3 close=0.15 or SKIP</t>
         </is>
       </c>
       <c r="B28">
-        <f>IF(LEN(Калькулятор!X2)&gt;20,"PASS","FAIL")</f>
+        <f>IF(StartLot&lt;&gt;2,"SKIP",IF(AND(CloseMode="THEORETICAL",ABS(Калькулятор!O4-0.15)&lt;1E-8),"PASS","FAIL"))</f>
         <v/>
       </c>
       <c r="C28">
@@ -2885,10 +2885,66 @@
         <v/>
       </c>
     </row>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>StartLot=2 L4 close=0.075 or SKIP</t>
+        </is>
+      </c>
+      <c r="B29">
+        <f>IF(StartLot&lt;&gt;2,"SKIP",IF(AND(CloseMode="THEORETICAL",ABS(Калькулятор!O5-0.075)&lt;1E-8),"PASS","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="C29">
+        <f>B29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>StartLot=2 L5 close=0.0375 or SKIP</t>
+        </is>
+      </c>
+      <c r="B30">
+        <f>IF(StartLot&lt;&gt;2,"SKIP",IF(AND(CloseMode="THEORETICAL",ABS(Калькулятор!O6-0.0375)&lt;1E-8),"PASS","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="C30">
+        <f>B30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Comment contains Big BUY or Big SELL</t>
+        </is>
+      </c>
+      <c r="B31">
+        <f>IF(OR(ISNUMBER(SEARCH("Big BUY",Калькулятор!X2)),ISNUMBER(SEARCH("Big SELL",Калькулятор!X2))),"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C31">
+        <f>B31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Comment not empty</t>
+        </is>
+      </c>
+      <c r="B32">
+        <f>IF(LEN(Калькулятор!X2)&gt;20,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="C32">
+        <f>B32</f>
+        <v/>
+      </c>
+    </row>
     <row r="33"/>
     <row r="34"/>
     <row r="35"/>

</xml_diff>